<commit_message>
Add Simon Willison blog post and solopreneur business architect playbook
Add Simon Willison's "Claude Code: Best Practices for Agentic Coding" blog post
and new solopreneur-business-architect playbook with template.

Co-Authored-By: Claude (claude-opus-4-6) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/Blog.xlsx
+++ b/src/Blog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="80.83203125" customWidth="1"/>
@@ -657,9 +657,44 @@
         <v>2026-02-07</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Claude Code: Best Practices for Agentic Coding</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Simon Willison breaks down Anthropic's best practices for Claude Code, revealing how 'think' trigger words map to different token budgets for extended reasoning.</v>
+      </c>
+      <c r="C8" t="str">
+        <v>guide</v>
+      </c>
+      <c r="D8" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E8" t="str">
+        <v>5</v>
+      </c>
+      <c r="F8" t="str">
+        <v>https://simonwillison.net/2025/Apr/19/claude-code-best-practices/</v>
+      </c>
+      <c r="G8" t="b">
+        <v>0</v>
+      </c>
+      <c r="H8" t="str">
+        <v>agent</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Best Practices</v>
+      </c>
+      <c r="J8" t="str">
+        <v>best practices; extended thinking; agentic coding; Simon Willison</v>
+      </c>
+      <c r="K8" t="str">
+        <v>2026-02-09</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add InfoQ article on Boris Cherny's Claude Code workflow
Add "Inside the Development Workflow of Claude Code's Creator" covering
parallel sessions, plan-then-execute, Opus 4.5, slash commands, and
verification loops.

Co-Authored-By: Claude (claude-opus-4-6) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/Blog.xlsx
+++ b/src/Blog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="80.83203125" customWidth="1"/>
@@ -692,9 +692,44 @@
         <v>2026-02-09</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Inside the Development Workflow of Claude Code's Creator</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Boris Cherny shares his 8-step Claude Code workflow including parallel sessions, plan-then-execute methodology, Opus 4.5 usage, slash commands, and verification loops that improve results 2-3x.</v>
+      </c>
+      <c r="C9" t="str">
+        <v>guide</v>
+      </c>
+      <c r="D9" t="str">
+        <v>advanced</v>
+      </c>
+      <c r="E9" t="str">
+        <v>8</v>
+      </c>
+      <c r="F9" t="str">
+        <v>https://www.infoq.com/news/2026/01/claude-code-creator-workflow/</v>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" t="str">
+        <v>agent</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Creator Workflow</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Boris Cherny; parallel sessions; plan mode; Opus 4.5; slash commands; CLAUDE.md</v>
+      </c>
+      <c r="K9" t="str">
+        <v>2026-02-10</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Puzzmo's 6 Weeks of Claude Code experience report
Add honest long-form review from Puzzmo's engineering lead covering
dual clone workflows, monorepo advantages, tech debt elimination,
and practical recommendations for experienced engineers.

Co-Authored-By: Claude (claude-opus-4-6) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/Blog.xlsx
+++ b/src/Blog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K10"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="80.83203125" customWidth="1"/>
@@ -727,9 +727,44 @@
         <v>2026-02-10</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>6 Weeks of Claude Code</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Puzzmo's engineering lead shares an honest 6-week experience report — completing years of tech debt as side projects, dual clone workflows, monorepo advantages, and why Claude Code works best as a pairing tool for experienced engineers.</v>
+      </c>
+      <c r="C10" t="str">
+        <v>guide</v>
+      </c>
+      <c r="D10" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E10" t="str">
+        <v>15</v>
+      </c>
+      <c r="F10" t="str">
+        <v>https://blog.puzzmo.com/posts/2025/07/30/six-weeks-of-claude-code/</v>
+      </c>
+      <c r="G10" t="b">
+        <v>0</v>
+      </c>
+      <c r="H10" t="str">
+        <v>agent</v>
+      </c>
+      <c r="I10" t="str">
+        <v>6 Week Review</v>
+      </c>
+      <c r="J10" t="str">
+        <v>experience report; tech debt; monorepo; parallel workflows; game dev; Puzzmo</v>
+      </c>
+      <c r="K10" t="str">
+        <v>2026-02-11</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add DEV Community article on Claude Code in production workflows
Add "Claude Code in Production: 40% Productivity Increase" covering
CLAUDE.md hierarchies, subagent code reviews, fast vs. full workflows,
and feature-based project organization with concrete metrics.

Co-Authored-By: Claude (claude-opus-4-6) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/Blog.xlsx
+++ b/src/Blog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K11"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="80.83203125" customWidth="1"/>
@@ -762,9 +762,44 @@
         <v>2026-02-11</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Claude Code in Production: 40% Productivity Increase</v>
+      </c>
+      <c r="B11" t="str">
+        <v>A solo developer maintaining 350k+ LOC documents a 40% productivity boost over 4 months with Claude Code — covering CLAUDE.md hierarchies, subagent code reviews, fast vs. full workflows, and feature-based project organization.</v>
+      </c>
+      <c r="C11" t="str">
+        <v>tutorial</v>
+      </c>
+      <c r="D11" t="str">
+        <v>advanced</v>
+      </c>
+      <c r="E11" t="str">
+        <v>12</v>
+      </c>
+      <c r="F11" t="str">
+        <v>https://dev.to/dzianiskarviha/integrating-claude-code-into-production-workflows-lbn</v>
+      </c>
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" t="str">
+        <v>agent</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Production Use</v>
+      </c>
+      <c r="J11" t="str">
+        <v>production workflows; CLAUDE.md; subagents; MCP; skills; code review; monorepo; productivity metrics</v>
+      </c>
+      <c r="K11" t="str">
+        <v>2026-02-12</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add final 4 blog posts completing the top 10 resources list
- Cooking with Claude Code: The Complete Guide (Sid Bharath)
- Google Engineer's Claude Code Confession (PPC Land)
- Claude Code is a Beast — Tips from 6 Months (DEV Community)
- Anthropic's Claude Code Transforms Vibe Coding (Axios)

Co-Authored-By: Claude (claude-opus-4-6) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/Blog.xlsx
+++ b/src/Blog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K15"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="80.83203125" customWidth="1"/>
@@ -797,9 +797,149 @@
         <v>2026-02-12</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Cooking with Claude Code: The Complete Guide</v>
+      </c>
+      <c r="B12" t="str">
+        <v>A continuously updated complete guide covering plugins, Chrome integration, sub-agents, MCP servers, slash commands, plan mode, git worktrees, and cloud teleporting — everything you need to use Claude Code as a full development partner.</v>
+      </c>
+      <c r="C12" t="str">
+        <v>guide</v>
+      </c>
+      <c r="D12" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E12" t="str">
+        <v>20</v>
+      </c>
+      <c r="F12" t="str">
+        <v>https://sidbharath.com/blog/claude-code-the-complete-guide/</v>
+      </c>
+      <c r="G12" t="b">
+        <v>0</v>
+      </c>
+      <c r="H12" t="str">
+        <v>skill</v>
+      </c>
+      <c r="I12" t="str">
+        <v>Complete Guide</v>
+      </c>
+      <c r="J12" t="str">
+        <v>complete guide; plugins; Chrome extension; sub-agents; MCP; slash commands; plan mode; git worktrees; teleporting</v>
+      </c>
+      <c r="K12" t="str">
+        <v>2026-02-13</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Google Engineer's Claude Code Confession Rattles Engineering Teams</v>
+      </c>
+      <c r="B13" t="str">
+        <v>A Google principal engineer reveals Claude Code replicated a year of distributed systems architecture in one hour — sparking a viral debate about organizational bottlenecks, knowledge amplification, and AI's role in cutting through bureaucracy.</v>
+      </c>
+      <c r="C13" t="str">
+        <v>news</v>
+      </c>
+      <c r="D13" t="str">
+        <v>basic</v>
+      </c>
+      <c r="E13" t="str">
+        <v>6</v>
+      </c>
+      <c r="F13" t="str">
+        <v>https://ppc.land/google-engineers-claude-code-confession-rattles-engineering-teams/</v>
+      </c>
+      <c r="G13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H13" t="str">
+        <v>default</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Viral Moment</v>
+      </c>
+      <c r="J13" t="str">
+        <v>Google; distributed systems; Paul Graham; viral; organizational bottlenecks; knowledge amplification</v>
+      </c>
+      <c r="K13" t="str">
+        <v>2026-02-13</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Claude Code is a Beast — Tips from 6 Months of Hardcore Use</v>
+      </c>
+      <c r="B14" t="str">
+        <v>A developer shares battle-tested tips from 6 months of intensive Claude Code use — auto-activating skills via hooks, dev docs workflow to prevent context loss, PM2 process management, specialized subagents, and a 100k to 400k LOC solo rewrite.</v>
+      </c>
+      <c r="C14" t="str">
+        <v>tutorial</v>
+      </c>
+      <c r="D14" t="str">
+        <v>advanced</v>
+      </c>
+      <c r="E14" t="str">
+        <v>14</v>
+      </c>
+      <c r="F14" t="str">
+        <v>https://dev.to/diet-code103/claude-code-is-a-beast-tips-from-6-months-of-hardcore-use-572n</v>
+      </c>
+      <c r="G14" t="b">
+        <v>0</v>
+      </c>
+      <c r="H14" t="str">
+        <v>agent</v>
+      </c>
+      <c r="I14" t="str">
+        <v>Power Tips</v>
+      </c>
+      <c r="J14" t="str">
+        <v>hooks; skills auto-activation; subagents; dev docs; PM2; context management; slash commands; SuperWhisper</v>
+      </c>
+      <c r="K14" t="str">
+        <v>2026-02-14</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Anthropic's Claude Code Transforms Vibe Coding</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Axios covers the cultural moment around Claude Code — how terminal-based agentic coding is changing who gets to build software, why the holiday break was a catalyst, and what separates prototyping from production-ready development.</v>
+      </c>
+      <c r="C15" t="str">
+        <v>news</v>
+      </c>
+      <c r="D15" t="str">
+        <v>basic</v>
+      </c>
+      <c r="E15" t="str">
+        <v>5</v>
+      </c>
+      <c r="F15" t="str">
+        <v>https://www.axios.com/2026/01/07/anthropics-claude-code-vibe-coding</v>
+      </c>
+      <c r="G15" t="b">
+        <v>0</v>
+      </c>
+      <c r="H15" t="str">
+        <v>default</v>
+      </c>
+      <c r="I15" t="str">
+        <v>Vibe Coding</v>
+      </c>
+      <c r="J15" t="str">
+        <v>vibe coding; mainstream media; Axios; cultural moment; terminal; agentic coding</v>
+      </c>
+      <c r="K15" t="str">
+        <v>2026-02-14</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K15"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Eyad Khrais tutorial blog post and X/Twitter Growth System playbook
- Blog: "The Complete Claude Code Tutorial" (viral 48M-view thread on
  skills, subagents, and MCP connectors)
- Playbook: x-twitter-growth-system with copy-paste template

Co-Authored-By: Claude (claude-opus-4-6) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/Blog.xlsx
+++ b/src/Blog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K16"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="80.83203125" customWidth="1"/>
@@ -937,9 +937,44 @@
         <v>2026-02-14</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>The Complete Claude Code Tutorial — Eyad Khrais</v>
+      </c>
+      <c r="B16" t="str">
+        <v>A viral 48M-view tutorial from ex-Amazon/Disney engineer Eyad Khrais breaking down Claude Code's three power features: Skills for encoding team patterns, Subagents for isolated task execution with fresh 200K context windows, and MCP connectors for eliminating tab-switching across GitHub, Slack, and databases.</v>
+      </c>
+      <c r="C16" t="str">
+        <v>tutorial</v>
+      </c>
+      <c r="D16" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E16" t="str">
+        <v>10</v>
+      </c>
+      <c r="F16" t="str">
+        <v>https://x.com/eyad_khrais/status/2010076957938188661</v>
+      </c>
+      <c r="G16" t="b">
+        <v>1</v>
+      </c>
+      <c r="H16" t="str">
+        <v>skill</v>
+      </c>
+      <c r="I16" t="str">
+        <v>Full Tutorial</v>
+      </c>
+      <c r="J16" t="str">
+        <v>skills; subagents; MCP; progressive disclosure; custom agents; tutorial; viral thread</v>
+      </c>
+      <c r="K16" t="str">
+        <v>2026-02-15</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Move Latest button to hero section and add new blog post
- Move Latest link from nav bar to hero quick links for better mobile layout
- Style Latest button with prominent orange border/bg to stand out
- Remove unused Sparkles import from layout
- Add "Top 10 Claude Code Tips for Non-Developers" blog post by JJ Englert

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/Blog.xlsx
+++ b/src/Blog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K17"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="80.83203125" customWidth="1"/>
@@ -972,9 +972,44 @@
         <v>2026-02-15</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Top 10 Claude Code Tips for Non-Developers</v>
+      </c>
+      <c r="B17" t="str">
+        <v>JJ Englert shares his top 10 tips for non-developers using Claude Code, drawn from building 20+ projects without writing a single line of code.</v>
+      </c>
+      <c r="C17" t="str">
+        <v>tutorial</v>
+      </c>
+      <c r="D17" t="str">
+        <v>basic</v>
+      </c>
+      <c r="E17" t="str">
+        <v>24</v>
+      </c>
+      <c r="F17" t="str">
+        <v>https://x.com/JJEnglert/status/2024858907773169874</v>
+      </c>
+      <c r="G17" t="b">
+        <v>1</v>
+      </c>
+      <c r="H17" t="str">
+        <v>agent</v>
+      </c>
+      <c r="I17" t="str">
+        <v>no-code tips</v>
+      </c>
+      <c r="J17" t="str">
+        <v>non-developer; tips; no-code; vibe coding; video; workflow</v>
+      </c>
+      <c r="K17" t="str">
+        <v>2026-02-20</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add blog post: Skills, Explained by Gabriel Chua
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/Blog.xlsx
+++ b/src/Blog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K18"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="80.83203125" customWidth="1"/>
@@ -1007,9 +1007,44 @@
         <v>2026-02-20</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Skills, Explained: Why Folders of Markdown Files Are So Effective</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Explores how AI skills — organized collections of prompts and resources in markdown files — let teams standardize recurring tasks through progressive disclosure, modular structure, and bundled resources.</v>
+      </c>
+      <c r="C18" t="str">
+        <v>guide</v>
+      </c>
+      <c r="D18" t="str">
+        <v>basic</v>
+      </c>
+      <c r="E18" t="str">
+        <v>8 min read</v>
+      </c>
+      <c r="F18" t="str">
+        <v>https://x.com/gabrielchua/status/2026687426593436066</v>
+      </c>
+      <c r="G18" t="b">
+        <v>0</v>
+      </c>
+      <c r="H18" t="str">
+        <v>skill</v>
+      </c>
+      <c r="I18" t="str">
+        <v>Skills</v>
+      </c>
+      <c r="J18" t="str">
+        <v>skills; markdown; prompting; workflows; agents; teams; codex</v>
+      </c>
+      <c r="K18" t="str">
+        <v>2026-02-25</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add blog post: The Shorthand Guide to Everything Claude Code
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/Blog.xlsx
+++ b/src/Blog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K19"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="80.83203125" customWidth="1"/>
@@ -1042,9 +1042,44 @@
         <v>2026-02-25</v>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>The Shorthand Guide to Everything Claude Code</v>
+      </c>
+      <c r="B19" t="str">
+        <v>A complete Claude Code setup guide after 10 months of daily use covering skills, hooks, subagents, MCPs, plugins, context window management, and practical tips.</v>
+      </c>
+      <c r="C19" t="str">
+        <v>guide</v>
+      </c>
+      <c r="D19" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E19" t="str">
+        <v>15</v>
+      </c>
+      <c r="F19" t="str">
+        <v>https://x.com/affaanmustafa/status/2012378465664745795</v>
+      </c>
+      <c r="G19" t="b">
+        <v>1</v>
+      </c>
+      <c r="H19" t="str">
+        <v>skill</v>
+      </c>
+      <c r="I19" t="str">
+        <v>complete setup</v>
+      </c>
+      <c r="J19" t="str">
+        <v>skills; hooks; subagents; mcp; plugins; context window; setup; configuration</v>
+      </c>
+      <c r="K19" t="str">
+        <v>2026-01-17</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K18"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add date display to blog posts and add Claude-Native Law Firm article
Show createdAt date on blog list items and carousel cards. Add new blog
post: "The Claude-Native Law Firm" by Zack Shapiro about practicing law
with Claude in 2026.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/Blog.xlsx
+++ b/src/Blog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K20"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="80.83203125" customWidth="1"/>
@@ -1077,9 +1077,44 @@
         <v>2026-01-17</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>The Claude-Native Law Firm — How I Actually Practice Law with AI in 2026</v>
+      </c>
+      <c r="B20" t="str">
+        <v>A practicing lawyer details how he runs a two-person boutique firm that competes with large firms by building his practice around Claude, using custom skills, autonomous cowork mode, and XML-level document manipulation for contract review, legal research, and real-time negotiation support.</v>
+      </c>
+      <c r="C20" t="str">
+        <v>guide</v>
+      </c>
+      <c r="D20" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E20" t="str">
+        <v>25 min read</v>
+      </c>
+      <c r="F20" t="str">
+        <v>https://x.com/zackbshapiro/status/2027389987444957625</v>
+      </c>
+      <c r="G20" t="b">
+        <v>0</v>
+      </c>
+      <c r="H20" t="str">
+        <v>skill</v>
+      </c>
+      <c r="I20" t="str">
+        <v>law firm</v>
+      </c>
+      <c r="J20" t="str">
+        <v>legal; AI workflows; skills; cowork; contract review; law; productivity</v>
+      </c>
+      <c r="K20" t="str">
+        <v>2026-03-06</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K20"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Cowork tutorial blog post and 11 content/marketing playbooks
New blog post: Claude Cowork Masterclass for Beginners (Full Tutorial)
New playbooks: audience-swipe-file, competitor-intelligence-brief,
content-drift-monitor, content-gap-finder, content-repurposer,
critic-agent, engagement-pattern-analyzer, follower-research-briefing,
funnel-metrics-analyst, trending-conversations-scout,
voice-of-customer-tracker — each with copy-paste templates.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/Blog.xlsx
+++ b/src/Blog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K21"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="80.83203125" customWidth="1"/>
@@ -1112,9 +1112,44 @@
         <v>2026-03-06</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Claude Cowork Masterclass for Beginners (Full Tutorial)</v>
+      </c>
+      <c r="B21" t="str">
+        <v>A comprehensive beginner's guide to Claude Cowork covering setup, context files, plugins, and real use cases for turning Claude into an autonomous coworker on your desktop.</v>
+      </c>
+      <c r="C21" t="str">
+        <v>tutorial</v>
+      </c>
+      <c r="D21" t="str">
+        <v>basic</v>
+      </c>
+      <c r="E21" t="str">
+        <v>8</v>
+      </c>
+      <c r="F21" t="str">
+        <v>https://x.com/coreyganim/status/2028470330247803361</v>
+      </c>
+      <c r="G21" t="b">
+        <v>0</v>
+      </c>
+      <c r="H21" t="str">
+        <v>agent</v>
+      </c>
+      <c r="I21" t="str">
+        <v>cowork guide</v>
+      </c>
+      <c r="J21" t="str">
+        <v>cowork; desktop; beginner; tutorial; automation; workspace; context files</v>
+      </c>
+      <c r="K21" t="str">
+        <v>2026-03-08</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add blog post: Everything Claude Code Can Do That You Haven't Tried Yet
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/Blog.xlsx
+++ b/src/Blog.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K22"/>
   <cols>
     <col min="1" max="1" width="60.83203125" customWidth="1"/>
     <col min="2" max="2" width="80.83203125" customWidth="1"/>
@@ -1147,9 +1147,44 @@
         <v>2026-03-08</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Everything Claude Code Can Do That You Haven't Tried Yet</v>
+      </c>
+      <c r="B22" t="str">
+        <v>A deep dive into five powerful but underused Claude Code features: Agent Skills, SessionStart Hooks, retroactive IaC with AWS CloudFormation, fixing context rot with GSD, and Google Workspace integration.</v>
+      </c>
+      <c r="C22" t="str">
+        <v>guide</v>
+      </c>
+      <c r="D22" t="str">
+        <v>intermediate</v>
+      </c>
+      <c r="E22" t="str">
+        <v>8</v>
+      </c>
+      <c r="F22" t="str">
+        <v>https://x.com/sharbel/status/2031372411283575012</v>
+      </c>
+      <c r="G22" t="b">
+        <v>1</v>
+      </c>
+      <c r="H22" t="str">
+        <v>agent</v>
+      </c>
+      <c r="I22" t="str">
+        <v>power features</v>
+      </c>
+      <c r="J22" t="str">
+        <v>agent skills; hooks; context rot; GSD; google workspace; AWS; CloudFormation; tips</v>
+      </c>
+      <c r="K22" t="str">
+        <v>2026-03-15</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>